<commit_message>
Update soccer trades 2026-08-14 00:04:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/La Liga/trades.xlsx
+++ b/data/sxbet/ligas/La Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
+          <t>0x11476693f9b725995aedcf0e75acf05d19a0f1647da3059f334da311f0f1e922</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1.19253</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0x10c92f089fb69109ac5beea7c82a0e1cd2f23257cd842348710e2598be68bc48</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786640471</t>
+          <t>1786664168</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>12.195122</t>
+          <t>2.08758</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
+          <t>0x046492cfcbf4e5a3ced4caa85326fa8b44dbff1fb248a61a7fa6c8a8d2d9c1f8</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>26.96</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -698,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xfcdcf41a0510583d5bb65df7215b5101ff435808043952db2a0364f1424743db</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786640450</t>
+          <t>1786663762</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>65.957187</t>
+          <t>8.385744</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,39 +739,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
+          <t>0xe376b22b83ba1a0d5c58e6763337d61f4445c85bfdc77949472d41c7c47e42b6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -795,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786639065</t>
+          <t>1786657450</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>36.891954</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +843,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
+          <t>0x4e949c2076e8faf4dcc272acfa8d69c62442324aca8ceeb5820b8348c74f13f6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,12 +858,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>16.42</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4213</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,7 +873,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -907,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786633518</t>
+          <t>1786657449</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>11.869436</t>
+          <t>52.967742</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,27 +955,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
+          <t>0xd54151c9cd066d8a5e7714f77ebc5e24ee2aac3e2c8a52a50b3a6becd0bac875</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>53.83</t>
+          <t>112.94</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1007,11 +979,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -1019,27 +987,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0x78a4cf6b02d047f006e2c80b80d1bba724ebd9a508d0cce70fc13d1dcc698bd3</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1064,17 +1032,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786633487</t>
+          <t>1786656774</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>128.166667</t>
+          <t>170.475472</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,28 +1059,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
+          <t>0x835c08ffc86c9c616d8c107e844ff9658b10b62372398122a4f7ded5bb28a516</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
+          <t>0x8e9bE2B8b636Cc98b01957cE9D4E3B62cF579080</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>72.15999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1123,27 +1091,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1136,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786632901</t>
+          <t>1786651844</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>120.26665</t>
+          <t>8.492552</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,28 +1163,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
+          <t>0x45cc84f2dd4c1b45226a895eead76c109d5af22eac83562ab8aa23758f8a6b5e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.1038</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1227,27 +1195,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Espanyol vs Levante</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19370489</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,17 +1240,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786631513</t>
+          <t>1786651814</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786899600</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>76.240964</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,28 +1267,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
+          <t>0x213398a7cadc42743f3aee31a89c45cc1f9c78136646bd816983864c34b13f79</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x4feB57379592eb94c51c014553de6EEbD4d42577</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1331,27 +1299,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1344,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786631323</t>
+          <t>1786651743</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>78.123457</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,28 +1371,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
+          <t>0x0adf7a0f94fb74bebb4e5acb49582e1f91e3ae462b204becaedfbe0f50714ede</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x06a603b688E676702ec63D735CAe4A57ff71B3e1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.11</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.165</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1435,27 +1403,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,17 +1448,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786631207</t>
+          <t>1786651718</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>67.333333</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,23 +1475,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
+          <t>0xc33e951dfa8d84c01759f86fe63dfc68ddc2b547988e3a32445d72b681f7f7a5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.85998</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.7113</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1539,27 +1507,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1584,17 +1552,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786630102</t>
+          <t>1786651637</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>16.67484</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,28 +1579,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
+          <t>0x948b3c3ece530e62252af65b92bdd73725833fe7355d5496ab1d4f6d84e43cc4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1643,27 +1611,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1688,17 +1656,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786626342</t>
+          <t>1786651588</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>11.331445</t>
+          <t>1.709402</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,28 +1683,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
+          <t>0x7578c65431424d3ae35de659ad6d246a7814cbb553d85319bf0968700f7bca4a</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16.18903</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1747,27 +1715,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1792,17 +1760,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786626327</t>
+          <t>1786651585</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>36.68902</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,28 +1787,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
+          <t>0x28bc2779df67c8165804579669b7a40ef9e3a34f89e4d9d4c81a44f6c49d8be2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x2F9aCBd9B89C6eF3bc3Dc2B0F0cCD0E0936BF912</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>35.45869</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2537</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1851,27 +1819,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1896,17 +1864,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786624561</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>139.73868</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,23 +1891,23 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
+          <t>0x0eaa76f318c30c9b01a36fedfdc1b48daafadd063ed5c90a74fd0908bdecfce3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x6203b6338991Ec84C8A8f5ef06bC17ceB1395Ddb</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.7163</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1955,27 +1923,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2000,17 +1968,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786623012</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>6.980803</t>
+          <t>11.965812</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2027,28 +1995,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
+          <t>0xcc54eb94d459bc0b9a34beb78c07fafbc7c1f3e7c6d43846f17fb20856c43d24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>28.91904</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.6038</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2059,27 +2027,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2104,17 +2072,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>47.899031</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2131,23 +2099,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
+          <t>0x1b14ab3ce842bb0ded035add24fcdd28a77380141c189ae36b1f623e70dff465</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>30.81465</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7113</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2163,27 +2131,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2208,17 +2176,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>43.32464</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2235,67 +2203,59 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
+          <t>0x31a8e64cfb4307b5b608318a4e037810f68fe9bef13258aa7d3c45dd664c0ad3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x03d4fFC791EE4A80194C9d9782E7D56407b242Ed</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>63.86</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4187</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>La Liga</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2320,17 +2280,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786621976</t>
+          <t>1786651558</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>152.501493</t>
+          <t>25.641026</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2347,39 +2307,31 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
+          <t>0x1c244dc1d052ae42a83bf5640bcba1b28bb9c28853e7f42713fa4fddcb66b677</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>97.87</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2387,27 +2339,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2432,17 +2384,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786651550</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>320.885246</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2459,12 +2411,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
+          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2474,22 +2426,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>82.86999</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.7363</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Racing Santander +1</t>
+          <t>Deportivo Alaves -0.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2499,27 +2451,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2544,17 +2496,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786640471</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>112.556862</t>
+          <t>12.195122</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2571,7 +2523,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
+          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2586,12 +2538,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>44.82</t>
+          <t>26.96</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2601,7 +2553,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Racing Santander -0.5</t>
+          <t>Deportivo Alaves -0.5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2611,27 +2563,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2656,17 +2608,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786640450</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>146.95082</t>
+          <t>65.957187</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2683,31 +2635,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
+          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>27.87224</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5325</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2715,27 +2675,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2760,17 +2720,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786619056</t>
+          <t>1786639065</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>52.342235</t>
+          <t>36.891954</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2787,12 +2747,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2802,12 +2762,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.4213</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2817,32 +2777,32 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
           <t>Rayo Vallecano</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Sevilla vs Rayo Vallecano</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Rayo Vallecano</t>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2872,7 +2832,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786614389</t>
+          <t>1786633518</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2882,7 +2842,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>175.438596</t>
+          <t>11.869436</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2899,12 +2859,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2914,22 +2874,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>53.83</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2939,27 +2899,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2984,17 +2944,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786586644</t>
+          <t>1786633487</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>7.769231</t>
+          <t>128.166667</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3011,28 +2971,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x27be56be09649bd460766fe27df249788cf4d7ad87d19f5f9a8bfba225e519b9</t>
+          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.52676</t>
+          <t>72.15999</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.7512</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3058,55 +3018,1975 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1786632901</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>120.26665</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>7.91</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.1038</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Espanyol vs Levante</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Espanyol</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19370489</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786631513</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786899600</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>76.240964</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>7.91</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.1013</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19370582</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786631323</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786822200</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>78.123457</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>11.11</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.165</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786631207</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>67.333333</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>11.85998</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.7113</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786630102</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>16.67484</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.4412</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1786626342</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>11.331445</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>16.18903</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4412</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1786626327</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>36.68902</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>35.45869</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.2537</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1786624561</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>139.73868</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.7163</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1786623012</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>6.980803</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>28.91904</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.6038</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1786622982</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>47.899031</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>30.81465</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.7113</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1786622982</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>43.32464</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>63.86</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.4187</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1786621976</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>152.501493</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>97.87</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.305</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>320.885246</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>82.86999</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.7363</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Racing Santander +1</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>112.556862</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>44.82</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.305</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Racing Santander -0.5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>146.95082</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>27.87224</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.5325</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Celta de Vigo vs Osasuna</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Celta de Vigo</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19370496</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1786619056</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1786908600</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>52.342235</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19370582</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1786614389</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1786822200</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>175.438596</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1786586644</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>7.769231</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0x27be56be09649bd460766fe27df249788cf4d7ad87d19f5f9a8bfba225e519b9</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1.52676</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.7512</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
           <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>L19370598</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
         <is>
           <t>1786578252</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>1786815000</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>2.032293</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-14 03:04:14 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/La Liga/trades.xlsx
+++ b/data/sxbet/ligas/La Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x11476693f9b725995aedcf0e75acf05d19a0f1647da3059f334da311f0f1e922</t>
+          <t>0xec715718ce1e06f5bfd1790eedf07c987dbe7e219a72c5facd15377495db5263</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.19253</t>
+          <t>122.1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5713</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x10c92f089fb69109ac5beea7c82a0e1cd2f23257cd842348710e2598be68bc48</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786664168</t>
+          <t>1786676253</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.08758</t>
+          <t>740.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,23 +635,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x046492cfcbf4e5a3ced4caa85326fa8b44dbff1fb248a61a7fa6c8a8d2d9c1f8</t>
+          <t>0x0e7729ad6b4a9824864f6ac006c58fb19124ac050b08faef247ac7a176fd96ee</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xB66Aa9923E7a8920151375e186E6718064dd4f08</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>245.05482</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.755</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xfcdcf41a0510583d5bb65df7215b5101ff435808043952db2a0364f1424743db</t>
+          <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786663762</t>
+          <t>1786669488</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>8.385744</t>
+          <t>324.575921</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,28 +739,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe376b22b83ba1a0d5c58e6763337d61f4445c85bfdc77949472d41c7c47e42b6</t>
+          <t>0x8d79a50b7331e59ea36d27efa5d99d53e26dfd1be15401e254a4cc43e280ff2f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+          <t>0x9737E0E3E8EE2DD6B8A7E19D1507EcB3221b5483</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>4.89999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.5863</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -771,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -816,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786657450</t>
+          <t>1786667446</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>8.358192</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,27 +843,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x4e949c2076e8faf4dcc272acfa8d69c62442324aca8ceeb5820b8348c74f13f6</t>
+          <t>0x11476693f9b725995aedcf0e75acf05d19a0f1647da3059f334da311f0f1e922</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16.42</t>
+          <t>1.19253</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -871,11 +867,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -883,27 +875,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0x10c92f089fb69109ac5beea7c82a0e1cd2f23257cd842348710e2598be68bc48</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,17 +920,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786657449</t>
+          <t>1786664168</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>52.967742</t>
+          <t>2.08758</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +947,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xd54151c9cd066d8a5e7714f77ebc5e24ee2aac3e2c8a52a50b3a6becd0bac875</t>
+          <t>0x046492cfcbf4e5a3ced4caa85326fa8b44dbff1fb248a61a7fa6c8a8d2d9c1f8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -966,12 +958,12 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>112.94</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1002,7 +994,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x78a4cf6b02d047f006e2c80b80d1bba724ebd9a508d0cce70fc13d1dcc698bd3</t>
+          <t>0xfcdcf41a0510583d5bb65df7215b5101ff435808043952db2a0364f1424743db</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1032,7 +1024,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786656774</t>
+          <t>1786663762</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1034,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>170.475472</t>
+          <t>8.385744</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,28 +1051,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x835c08ffc86c9c616d8c107e844ff9658b10b62372398122a4f7ded5bb28a516</t>
+          <t>0xe376b22b83ba1a0d5c58e6763337d61f4445c85bfdc77949472d41c7c47e42b6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8e9bE2B8b636Cc98b01957cE9D4E3B62cF579080</t>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5888</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1091,27 +1083,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1136,17 +1128,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786651844</t>
+          <t>1786657450</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>8.492552</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,31 +1155,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x45cc84f2dd4c1b45226a895eead76c109d5af22eac83562ab8aa23758f8a6b5e</t>
+          <t>0x4e949c2076e8faf4dcc272acfa8d69c62442324aca8ceeb5820b8348c74f13f6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>16.42</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1240,17 +1240,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786651814</t>
+          <t>1786657449</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>42.735043</t>
+          <t>52.967742</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1267,23 +1267,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x213398a7cadc42743f3aee31a89c45cc1f9c78136646bd816983864c34b13f79</t>
+          <t>0xd54151c9cd066d8a5e7714f77ebc5e24ee2aac3e2c8a52a50b3a6becd0bac875</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x4feB57379592eb94c51c014553de6EEbD4d42577</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>112.94</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1299,27 +1299,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0x78a4cf6b02d047f006e2c80b80d1bba724ebd9a508d0cce70fc13d1dcc698bd3</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786651743</t>
+          <t>1786656774</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>170.475472</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1371,12 +1371,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x0adf7a0f94fb74bebb4e5acb49582e1f91e3ae462b204becaedfbe0f50714ede</t>
+          <t>0x835c08ffc86c9c616d8c107e844ff9658b10b62372398122a4f7ded5bb28a516</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x06a603b688E676702ec63D735CAe4A57ff71B3e1</t>
+          <t>0x8e9bE2B8b636Cc98b01957cE9D4E3B62cF579080</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786651718</t>
+          <t>1786651844</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>8.492552</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1475,18 +1475,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xc33e951dfa8d84c01759f86fe63dfc68ddc2b547988e3a32445d72b681f7f7a5</t>
+          <t>0x45cc84f2dd4c1b45226a895eead76c109d5af22eac83562ab8aa23758f8a6b5e</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786651637</t>
+          <t>1786651814</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1579,28 +1579,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x948b3c3ece530e62252af65b92bdd73725833fe7355d5496ab1d4f6d84e43cc4</t>
+          <t>0x213398a7cadc42743f3aee31a89c45cc1f9c78136646bd816983864c34b13f79</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
+          <t>0x4feB57379592eb94c51c014553de6EEbD4d42577</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1611,27 +1611,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1656,17 +1656,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786651588</t>
+          <t>1786651743</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.709402</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1683,18 +1683,18 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x7578c65431424d3ae35de659ad6d246a7814cbb553d85319bf0968700f7bca4a</t>
+          <t>0x0adf7a0f94fb74bebb4e5acb49582e1f91e3ae462b204becaedfbe0f50714ede</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+          <t>0x06a603b688E676702ec63D735CAe4A57ff71B3e1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786651585</t>
+          <t>1786651718</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>17.094</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1787,18 +1787,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x28bc2779df67c8165804579669b7a40ef9e3a34f89e4d9d4c81a44f6c49d8be2</t>
+          <t>0xc33e951dfa8d84c01759f86fe63dfc68ddc2b547988e3a32445d72b681f7f7a5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x2F9aCBd9B89C6eF3bc3Dc2B0F0cCD0E0936BF912</t>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786651567</t>
+          <t>1786651637</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>17.094</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1891,18 +1891,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x0eaa76f318c30c9b01a36fedfdc1b48daafadd063ed5c90a74fd0908bdecfce3</t>
+          <t>0x948b3c3ece530e62252af65b92bdd73725833fe7355d5496ab1d4f6d84e43cc4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x6203b6338991Ec84C8A8f5ef06bC17ceB1395Ddb</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786651567</t>
+          <t>1786651588</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>11.965812</t>
+          <t>1.709402</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1995,18 +1995,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xcc54eb94d459bc0b9a34beb78c07fafbc7c1f3e7c6d43846f17fb20856c43d24</t>
+          <t>0x7578c65431424d3ae35de659ad6d246a7814cbb553d85319bf0968700f7bca4a</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786651559</t>
+          <t>1786651585</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>42.735043</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2099,12 +2099,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x1b14ab3ce842bb0ded035add24fcdd28a77380141c189ae36b1f623e70dff465</t>
+          <t>0x28bc2779df67c8165804579669b7a40ef9e3a34f89e4d9d4c81a44f6c49d8be2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+          <t>0x2F9aCBd9B89C6eF3bc3Dc2B0F0cCD0E0936BF912</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786651559</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2203,18 +2203,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x31a8e64cfb4307b5b608318a4e037810f68fe9bef13258aa7d3c45dd664c0ad3</t>
+          <t>0x0eaa76f318c30c9b01a36fedfdc1b48daafadd063ed5c90a74fd0908bdecfce3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x03d4fFC791EE4A80194C9d9782E7D56407b242Ed</t>
+          <t>0x6203b6338991Ec84C8A8f5ef06bC17ceB1395Ddb</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786651558</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>25.641026</t>
+          <t>11.965812</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2307,18 +2307,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x1c244dc1d052ae42a83bf5640bcba1b28bb9c28853e7f42713fa4fddcb66b677</t>
+          <t>0xcc54eb94d459bc0b9a34beb78c07fafbc7c1f3e7c6d43846f17fb20856c43d24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786651550</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2411,39 +2411,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
+          <t>0x1b14ab3ce842bb0ded035add24fcdd28a77380141c189ae36b1f623e70dff465</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2451,27 +2443,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2496,17 +2488,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786640471</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>12.195122</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2523,39 +2515,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
+          <t>0x31a8e64cfb4307b5b608318a4e037810f68fe9bef13258aa7d3c45dd664c0ad3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x03d4fFC791EE4A80194C9d9782E7D56407b242Ed</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>26.96</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2563,27 +2547,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2608,17 +2592,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786640450</t>
+          <t>1786651558</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>65.957187</t>
+          <t>25.641026</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2635,27 +2619,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
+          <t>0x1c244dc1d052ae42a83bf5640bcba1b28bb9c28853e7f42713fa4fddcb66b677</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2663,11 +2643,7 @@
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2675,27 +2651,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2720,17 +2696,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786639065</t>
+          <t>1786651550</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>36.891954</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2747,7 +2723,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
+          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2767,17 +2743,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4213</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves -0.5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2787,27 +2763,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2832,17 +2808,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786633518</t>
+          <t>1786640471</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>11.869436</t>
+          <t>12.195122</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2859,7 +2835,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
+          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2874,22 +2850,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>53.83</t>
+          <t>26.96</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves -0.5</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2899,27 +2875,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2944,17 +2920,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786633487</t>
+          <t>1786640450</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>128.166667</t>
+          <t>65.957187</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2971,31 +2947,39 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
+          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>72.15999</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3003,27 +2987,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3048,17 +3032,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786632901</t>
+          <t>1786639065</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>120.26665</t>
+          <t>36.891954</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3075,31 +3059,39 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
+          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.1038</t>
+          <t>1.4213</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3107,27 +3099,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Espanyol vs Levante</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19370489</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3152,17 +3144,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786631513</t>
+          <t>1786633518</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786899600</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>76.240964</t>
+          <t>11.869436</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3179,31 +3171,39 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
+          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>53.83</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786631323</t>
+          <t>1786633487</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>78.123457</t>
+          <t>128.166667</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3283,28 +3283,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
+          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>11.11</t>
+          <t>72.15999</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.165</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786631207</t>
+          <t>1786632901</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>67.333333</t>
+          <t>120.26665</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
+          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3398,17 +3398,17 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11.85998</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.7113</t>
+          <t>1.1038</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -3419,27 +3419,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Espanyol vs Levante</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370489</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3464,17 +3464,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786630102</t>
+          <t>1786631513</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786899600</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>16.67484</t>
+          <t>76.240964</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3491,28 +3491,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
+          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -3523,27 +3523,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3568,17 +3568,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786626342</t>
+          <t>1786631323</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>11.331445</t>
+          <t>78.123457</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3595,28 +3595,28 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
+          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>16.18903</t>
+          <t>11.11</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786626327</t>
+          <t>1786631207</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>36.68902</t>
+          <t>67.333333</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3699,28 +3699,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
+          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>35.45869</t>
+          <t>11.85998</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.2537</t>
+          <t>1.7113</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786624561</t>
+          <t>1786630102</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>139.73868</t>
+          <t>16.67484</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3803,7 +3803,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
+          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3819,12 +3819,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7163</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786623012</t>
+          <t>1786626342</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>6.980803</t>
+          <t>11.331445</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3907,7 +3907,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
+          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3918,17 +3918,17 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>28.91904</t>
+          <t>16.18903</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.6038</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786626327</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>47.899031</t>
+          <t>36.68902</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4011,7 +4011,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
+          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4022,17 +4022,17 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>30.81465</t>
+          <t>35.45869</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.7113</t>
+          <t>1.2537</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786624561</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>43.32464</t>
+          <t>139.73868</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4115,67 +4115,59 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
+          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>63.86</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.4187</t>
+          <t>1.7163</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>La Liga</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4200,17 +4192,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786621976</t>
+          <t>1786623012</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>152.501493</t>
+          <t>6.980803</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4227,7 +4219,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
+          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4235,31 +4227,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>97.87</t>
+          <t>28.91904</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.6038</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4267,27 +4251,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
+          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4312,17 +4296,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786622982</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>320.885246</t>
+          <t>47.899031</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4339,7 +4323,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
+          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4347,31 +4331,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>82.86999</t>
+          <t>30.81465</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.7363</t>
+          <t>1.7113</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Racing Santander +1</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4379,27 +4355,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4424,17 +4400,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786622982</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>112.556862</t>
+          <t>43.32464</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4451,7 +4427,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
+          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4466,22 +4442,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>44.82</t>
+          <t>63.86</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.4187</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>La Liga</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Racing Santander -0.5</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4506,7 +4482,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
+          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4536,7 +4512,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786621976</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4546,7 +4522,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>146.95082</t>
+          <t>152.501493</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4563,7 +4539,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
+          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4571,15 +4547,19 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>27.87224</t>
+          <t>97.87</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.5325</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4587,7 +4567,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4595,27 +4579,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4640,17 +4624,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786619056</t>
+          <t>1786621975</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>52.342235</t>
+          <t>320.885246</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4667,12 +4651,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4682,22 +4666,22 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>82.86999</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.7363</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Racing Santander +1</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -4707,27 +4691,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4752,17 +4736,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786614389</t>
+          <t>1786621975</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>175.438596</t>
+          <t>112.556862</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4779,12 +4763,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4794,22 +4778,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>44.82</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Racing Santander -0.5</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4819,27 +4803,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4864,17 +4848,17 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786586644</t>
+          <t>1786621975</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>7.769231</t>
+          <t>146.95082</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4891,23 +4875,23 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x27be56be09649bd460766fe27df249788cf4d7ad87d19f5f9a8bfba225e519b9</t>
+          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.52676</t>
+          <t>27.87224</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.7512</t>
+          <t>1.5325</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4923,70 +4907,398 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
+          <t>Celta de Vigo vs Osasuna</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Celta de Vigo</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19370496</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1786619056</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1786908600</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>52.342235</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19370582</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1786614389</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1786822200</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>175.438596</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
           <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Deportivo Alaves</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Getafe</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1786586644</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>7.769231</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0x27be56be09649bd460766fe27df249788cf4d7ad87d19f5f9a8bfba225e519b9</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1.52676</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.7512</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>L19370598</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
         <is>
           <t>1786578252</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>1786815000</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>2.032293</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-14 07:04:20 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/La Liga/trades.xlsx
+++ b/data/sxbet/ligas/La Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xec715718ce1e06f5bfd1790eedf07c987dbe7e219a72c5facd15377495db5263</t>
+          <t>0xbf1a151f615bf3f9a9e616e3c50bbe9cfcae4e7a99f9ce723f49c93c83cdc9d0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
+          <t>0x30E3f83573EbFc7274EeAfD586D930F7392F5650</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>122.1</t>
+          <t>1.16999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.165</t>
+          <t>1.5875</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786676253</t>
+          <t>1786687820</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>740.0</t>
+          <t>1.991472</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,23 +635,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x0e7729ad6b4a9824864f6ac006c58fb19124ac050b08faef247ac7a176fd96ee</t>
+          <t>0x11994251df996a13dca305742c6cfa502ae27aa5f4bd0111f29dc7341166926a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xB66Aa9923E7a8920151375e186E6718064dd4f08</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xdFC5342F5d4bF9F317c0CBf71121AC6FA92d8fbf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>245.05482</t>
+          <t>45.715</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.755</t>
+          <t>1.2788</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -659,7 +663,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
+          <t>0x9993d963f79cc9f688d38136ed8af60ad8c5e128ae668d0af49645c4ec2e0c25</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786669488</t>
+          <t>1786684730</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>324.575921</t>
+          <t>164.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,28 +747,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x8d79a50b7331e59ea36d27efa5d99d53e26dfd1be15401e254a4cc43e280ff2f</t>
+          <t>0x03eaa48ad5cba7703834b4eb4188b2512fc59fc66ce1a132f347fb208e62190e</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x9737E0E3E8EE2DD6B8A7E19D1507EcB3221b5483</t>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.89999</t>
+          <t>29.16362</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5863</t>
+          <t>1.1075</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -786,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786667446</t>
+          <t>1786684614</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>8.358192</t>
+          <t>271.289488</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,28 +851,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x11476693f9b725995aedcf0e75acf05d19a0f1647da3059f334da311f0f1e922</t>
+          <t>0xf7320171cfa1d2a4388cf7700c275208ec77d1f0986bae7466346769cb38d5b4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.19253</t>
+          <t>1.05797</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5713</t>
+          <t>1.1075</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -875,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x10c92f089fb69109ac5beea7c82a0e1cd2f23257cd842348710e2598be68bc48</t>
+          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -920,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786664168</t>
+          <t>1786684161</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2.08758</t>
+          <t>9.841581</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,28 +955,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x046492cfcbf4e5a3ced4caa85326fa8b44dbff1fb248a61a7fa6c8a8d2d9c1f8</t>
+          <t>0x2c667f7cd0a5ee4597a318320db656e61b2fe595b68044cdbb02a35a2c508f11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>122.1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -994,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xfcdcf41a0510583d5bb65df7215b5101ff435808043952db2a0364f1424743db</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1024,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786663762</t>
+          <t>1786679771</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1034,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>8.385744</t>
+          <t>740.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1051,28 +1059,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xe376b22b83ba1a0d5c58e6763337d61f4445c85bfdc77949472d41c7c47e42b6</t>
+          <t>0xef898b845c993efce01f949a5b4165e91083d76283cd50b5ccb38113072d39a3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>122.1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1083,27 +1091,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1128,17 +1136,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786657450</t>
+          <t>1786677944</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>740.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1155,39 +1163,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x4e949c2076e8faf4dcc272acfa8d69c62442324aca8ceeb5820b8348c74f13f6</t>
+          <t>0xec715718ce1e06f5bfd1790eedf07c987dbe7e219a72c5facd15377495db5263</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xf3F25e96ea1eb0FC87b1778eD6C76af72405e9a4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>16.42</t>
+          <t>122.1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1240,17 +1240,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786657449</t>
+          <t>1786676253</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>52.967742</t>
+          <t>740.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1267,23 +1267,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xd54151c9cd066d8a5e7714f77ebc5e24ee2aac3e2c8a52a50b3a6becd0bac875</t>
+          <t>0x0e7729ad6b4a9824864f6ac006c58fb19124ac050b08faef247ac7a176fd96ee</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xB66Aa9923E7a8920151375e186E6718064dd4f08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>112.94</t>
+          <t>245.05482</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.755</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x78a4cf6b02d047f006e2c80b80d1bba724ebd9a508d0cce70fc13d1dcc698bd3</t>
+          <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786656774</t>
+          <t>1786669488</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>170.475472</t>
+          <t>324.575921</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1371,23 +1371,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x835c08ffc86c9c616d8c107e844ff9658b10b62372398122a4f7ded5bb28a516</t>
+          <t>0x8d79a50b7331e59ea36d27efa5d99d53e26dfd1be15401e254a4cc43e280ff2f</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8e9bE2B8b636Cc98b01957cE9D4E3B62cF579080</t>
+          <t>0x9737E0E3E8EE2DD6B8A7E19D1507EcB3221b5483</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>4.89999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5888</t>
+          <t>1.5863</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786651844</t>
+          <t>1786667446</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>8.492552</t>
+          <t>8.358192</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1475,28 +1475,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x45cc84f2dd4c1b45226a895eead76c109d5af22eac83562ab8aa23758f8a6b5e</t>
+          <t>0x11476693f9b725995aedcf0e75acf05d19a0f1647da3059f334da311f0f1e922</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1.19253</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1507,27 +1507,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0x10c92f089fb69109ac5beea7c82a0e1cd2f23257cd842348710e2598be68bc48</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1552,17 +1552,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786651814</t>
+          <t>1786664168</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>42.735043</t>
+          <t>2.08758</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1579,23 +1579,23 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x213398a7cadc42743f3aee31a89c45cc1f9c78136646bd816983864c34b13f79</t>
+          <t>0x046492cfcbf4e5a3ced4caa85326fa8b44dbff1fb248a61a7fa6c8a8d2d9c1f8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x4feB57379592eb94c51c014553de6EEbD4d42577</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1611,27 +1611,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
+          <t>0xfcdcf41a0510583d5bb65df7215b5101ff435808043952db2a0364f1424743db</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1656,17 +1656,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786651743</t>
+          <t>1786663762</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>8.385744</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1683,28 +1683,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x0adf7a0f94fb74bebb4e5acb49582e1f91e3ae462b204becaedfbe0f50714ede</t>
+          <t>0xe376b22b83ba1a0d5c58e6763337d61f4445c85bfdc77949472d41c7c47e42b6</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x06a603b688E676702ec63D735CAe4A57ff71B3e1</t>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1715,27 +1715,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1760,17 +1760,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786651718</t>
+          <t>1786657450</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1787,31 +1787,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xc33e951dfa8d84c01759f86fe63dfc68ddc2b547988e3a32445d72b681f7f7a5</t>
+          <t>0x4e949c2076e8faf4dcc272acfa8d69c62442324aca8ceeb5820b8348c74f13f6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0xE4DD6165bFF7EE73D7932C3b478f7E22431e85E7</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>16.42</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -1819,27 +1827,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1864,17 +1872,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786651637</t>
+          <t>1786657449</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>52.967742</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1891,28 +1899,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x948b3c3ece530e62252af65b92bdd73725833fe7355d5496ab1d4f6d84e43cc4</t>
+          <t>0xd54151c9cd066d8a5e7714f77ebc5e24ee2aac3e2c8a52a50b3a6becd0bac875</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>112.94</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1923,27 +1931,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0x78a4cf6b02d047f006e2c80b80d1bba724ebd9a508d0cce70fc13d1dcc698bd3</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1968,17 +1976,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786651588</t>
+          <t>1786656774</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.709402</t>
+          <t>170.475472</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1995,23 +2003,23 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x7578c65431424d3ae35de659ad6d246a7814cbb553d85319bf0968700f7bca4a</t>
+          <t>0x835c08ffc86c9c616d8c107e844ff9658b10b62372398122a4f7ded5bb28a516</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+          <t>0x8e9bE2B8b636Cc98b01957cE9D4E3B62cF579080</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.5888</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2072,7 +2080,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786651585</t>
+          <t>1786651844</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2082,7 +2090,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>17.094</t>
+          <t>8.492552</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2099,18 +2107,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x28bc2779df67c8165804579669b7a40ef9e3a34f89e4d9d4c81a44f6c49d8be2</t>
+          <t>0x45cc84f2dd4c1b45226a895eead76c109d5af22eac83562ab8aa23758f8a6b5e</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x2F9aCBd9B89C6eF3bc3Dc2B0F0cCD0E0936BF912</t>
+          <t>0xa3786b93377213A42Bf1d3261d373cE67Cf2AA67</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2176,7 +2184,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786651567</t>
+          <t>1786651814</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2186,7 +2194,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>17.094</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2203,28 +2211,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x0eaa76f318c30c9b01a36fedfdc1b48daafadd063ed5c90a74fd0908bdecfce3</t>
+          <t>0x213398a7cadc42743f3aee31a89c45cc1f9c78136646bd816983864c34b13f79</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x6203b6338991Ec84C8A8f5ef06bC17ceB1395Ddb</t>
+          <t>0x4feB57379592eb94c51c014553de6EEbD4d42577</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.585</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2235,27 +2243,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Celta de Vigo vs Osasuna</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Celta de Vigo</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
+          <t>0xaf77554314e04318c5e0efc781f967e8d177d3d17ef168bc65dd3721e2dedc30</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370496</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2280,17 +2288,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786651567</t>
+          <t>1786651743</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786908600</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>11.965812</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2307,18 +2315,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcc54eb94d459bc0b9a34beb78c07fafbc7c1f3e7c6d43846f17fb20856c43d24</t>
+          <t>0x0adf7a0f94fb74bebb4e5acb49582e1f91e3ae462b204becaedfbe0f50714ede</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+          <t>0x06a603b688E676702ec63D735CAe4A57ff71B3e1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2384,7 +2392,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786651559</t>
+          <t>1786651718</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2394,7 +2402,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>42.735043</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2411,18 +2419,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x1b14ab3ce842bb0ded035add24fcdd28a77380141c189ae36b1f623e70dff465</t>
+          <t>0xc33e951dfa8d84c01759f86fe63dfc68ddc2b547988e3a32445d72b681f7f7a5</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.99999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2488,7 +2496,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786651559</t>
+          <t>1786651637</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2498,7 +2506,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>17.094</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2515,18 +2523,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x31a8e64cfb4307b5b608318a4e037810f68fe9bef13258aa7d3c45dd664c0ad3</t>
+          <t>0x948b3c3ece530e62252af65b92bdd73725833fe7355d5496ab1d4f6d84e43cc4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x03d4fFC791EE4A80194C9d9782E7D56407b242Ed</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2592,7 +2600,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786651558</t>
+          <t>1786651588</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2602,7 +2610,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>25.641026</t>
+          <t>1.709402</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2619,18 +2627,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x1c244dc1d052ae42a83bf5640bcba1b28bb9c28853e7f42713fa4fddcb66b677</t>
+          <t>0x7578c65431424d3ae35de659ad6d246a7814cbb553d85319bf0968700f7bca4a</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2696,7 +2704,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786651550</t>
+          <t>1786651585</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2706,7 +2714,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>8.546991</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2723,39 +2731,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
+          <t>0x28bc2779df67c8165804579669b7a40ef9e3a34f89e4d9d4c81a44f6c49d8be2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x2F9aCBd9B89C6eF3bc3Dc2B0F0cCD0E0936BF912</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2763,27 +2763,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2808,17 +2808,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786640471</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>12.195122</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2835,39 +2835,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
+          <t>0x0eaa76f318c30c9b01a36fedfdc1b48daafadd063ed5c90a74fd0908bdecfce3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x6203b6338991Ec84C8A8f5ef06bC17ceB1395Ddb</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>26.96</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Deportivo Alaves -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2875,27 +2867,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2920,17 +2912,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786640450</t>
+          <t>1786651567</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>65.957187</t>
+          <t>11.965812</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2947,27 +2939,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
+          <t>0xcc54eb94d459bc0b9a34beb78c07fafbc7c1f3e7c6d43846f17fb20856c43d24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>20.06</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2975,11 +2963,7 @@
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -2987,27 +2971,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3032,17 +3016,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786639065</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>36.891954</t>
+          <t>42.735043</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3059,54 +3043,46 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
+          <t>0x1b14ab3ce842bb0ded035add24fcdd28a77380141c189ae36b1f623e70dff465</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9.99999</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4213</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Sevilla vs Rayo Vallecano</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Rayo Vallecano</t>
@@ -3114,7 +3090,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3144,7 +3120,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786633518</t>
+          <t>1786651559</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3154,7 +3130,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>11.869436</t>
+          <t>17.094</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3171,54 +3147,46 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
+          <t>0x31a8e64cfb4307b5b608318a4e037810f68fe9bef13258aa7d3c45dd664c0ad3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x03d4fFC791EE4A80194C9d9782E7D56407b242Ed</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>53.83</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Sevilla</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Sevilla vs Rayo Vallecano</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Rayo Vallecano</t>
@@ -3226,7 +3194,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3256,7 +3224,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786633487</t>
+          <t>1786651558</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3266,7 +3234,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>128.166667</t>
+          <t>25.641026</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3283,28 +3251,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
+          <t>0x1c244dc1d052ae42a83bf5640bcba1b28bb9c28853e7f42713fa4fddcb66b677</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>72.15999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3315,27 +3283,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
+          <t>0xeb4881400081231ce3e5f9992ac7e23e85fe6e1fdfec6a3997b442a83b7307b1</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3360,17 +3328,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786632901</t>
+          <t>1786651550</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>120.26665</t>
+          <t>8.546991</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3387,31 +3355,39 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
+          <t>0x20fcd5dbfafe538f08c15c6b35af5d546fa35aa588ef9811c9696ac39843c736</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.1038</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves -0.5</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3419,27 +3395,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Espanyol vs Levante</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19370489</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3464,17 +3440,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786631513</t>
+          <t>1786640471</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786899600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>76.240964</t>
+          <t>12.195122</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3491,31 +3467,39 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
+          <t>0x48d06bf1eb103be3b93f605ad7b9ed301f228fa4dfae557dca83434f1d5e0c1a</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>26.96</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves -0.5</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3523,27 +3507,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3568,17 +3552,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786631323</t>
+          <t>1786640450</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>78.123457</t>
+          <t>65.957187</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3595,7 +3579,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
+          <t>0xe750c1fb5c3ef7edfc166b18659be46b00e3cc96d5ae299b162166175d07245f</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3603,23 +3587,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>11.11</t>
+          <t>20.06</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.165</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3627,27 +3619,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
+          <t>0x0a08c3d7f08812839b48fc67d5842cc07f2a5e67ce2a26c46d0210680fda2f99</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3672,17 +3664,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786631207</t>
+          <t>1786639065</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>67.333333</t>
+          <t>36.891954</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3699,31 +3691,39 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
+          <t>0xdc16a40eba6eeb7462531fd3b01240a8f58f0ea20568efbaba25b17131094f2e</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>11.85998</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.7113</t>
+          <t>1.4213</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3731,27 +3731,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3776,17 +3776,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786630102</t>
+          <t>1786633518</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>16.67484</t>
+          <t>11.869436</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3803,31 +3803,39 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
+          <t>0x1b67e861f8e383798d979684797f608bfad6122cc87844f2a37a8cf06e019030</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>53.83</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -3835,27 +3843,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0xa5db2f6f922d69f99abed1f24ad7fa38777c90f51d489e3c1aa07c74dddb10e0</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3880,17 +3888,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786626342</t>
+          <t>1786633487</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>11.331445</t>
+          <t>128.166667</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3907,28 +3915,28 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
+          <t>0x909a230aebd5eb00de6012a0eb69301784b515acf69e93ee497d243bd3ce212f</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xbcD65d7e2D58b95Cf434eB65a82b9FD5b682D144</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>16.18903</t>
+          <t>72.15999</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -3954,7 +3962,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
+          <t>0x1b8dfbd894484bd763d2600e4505a21a73c3b4cb8a3004a1654ba87980dbc559</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3984,7 +3992,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786626327</t>
+          <t>1786632901</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3994,7 +4002,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>36.68902</t>
+          <t>120.26665</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4011,28 +4019,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
+          <t>0x081a76991e0701cf3dbcaa6ccbdd7d9dd69242e812c8b7e977517fe836423751</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>35.45869</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.2537</t>
+          <t>1.1038</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -4043,27 +4051,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Espanyol vs Levante</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
+          <t>0xd36fc2a623f22222f73350186e7d08c0d31b2d895ac24a68dc8408d4e98bf55a</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370489</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4088,17 +4096,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786624561</t>
+          <t>1786631513</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786899600</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>139.73868</t>
+          <t>76.240964</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4115,28 +4123,28 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
+          <t>0x6f1c770a5b9534dbfff85f398a28d171effe0e02699c6558a37a881468f3090e</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.7163</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -4147,27 +4155,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Sevilla vs Rayo Vallecano</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
+          <t>0x3b99901d045414f7d5a55497712a0a61ef0f6a829783277b6f0583659a40517f</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370582</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4192,17 +4200,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786623012</t>
+          <t>1786631323</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786822200</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>6.980803</t>
+          <t>78.123457</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4219,28 +4227,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
+          <t>0xffde28cdfe7ae2b6324278e8117e605bc5c2ecb236877e683d06b5cbe620b2b1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>28.91904</t>
+          <t>11.11</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.6038</t>
+          <t>1.165</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4266,7 +4274,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
+          <t>0xdae71376e09c91d710d729fe77ea2e842f603f91974aa4731f913be7021c5796</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4296,7 +4304,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786631207</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4306,7 +4314,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>47.899031</t>
+          <t>67.333333</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4323,18 +4331,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
+          <t>0x1542e94d97dca7a28f2bf2b946f64e1fefc9fc04f50a7622a8a2791d01c58796</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>30.81465</t>
+          <t>11.85998</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4400,7 +4408,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786622982</t>
+          <t>1786630102</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4410,7 +4418,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>43.32464</t>
+          <t>16.67484</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4427,67 +4435,59 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
+          <t>0x9ff18d48c5ac1507ef9b6a3dfaf34f20966e85ee30cbd99e0df47a940abf1d32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>63.86</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.4187</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>La Liga</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>La Liga</t>
-        </is>
-      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4512,17 +4512,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786621976</t>
+          <t>1786626342</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>152.501493</t>
+          <t>11.331445</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4539,7 +4539,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
+          <t>0x50f0b3572b92fd4a3268a217b75ca6b4a52b72077d0276df9d0d123d8b3ebc60</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4547,31 +4547,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>97.87</t>
+          <t>16.18903</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Racing Santander</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4579,27 +4571,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
+          <t>0x776caca6c8b9cb32d9a7b2ec2b4f40bbb630001b4db7c24175062af09044b7dd</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4624,17 +4616,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786626327</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>320.885246</t>
+          <t>36.68902</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4651,7 +4643,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
+          <t>0x2d1550913dec85439afda8d85c6033895212998f22943ab968dee5cbd7d7e7a2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4659,31 +4651,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>82.86999</t>
+          <t>35.45869</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.7363</t>
+          <t>1.2537</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Racing Santander +1</t>
-        </is>
-      </c>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4691,27 +4675,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
+          <t>0x0596e7ef887839f51f014583ff32fca0dbfab0916b17c3d05d740985b59eabc3</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4736,17 +4720,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786624561</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>112.556862</t>
+          <t>139.73868</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4763,39 +4747,31 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
+          <t>0x6f809dd95ba0a7f41584a66e0979cb2c04ebaeefb6e5d949b0bfd9c53278c063</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>44.82</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.7163</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Racing Santander -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -4803,27 +4779,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Racing Santander vs Villarreal</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Racing Santander</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>L19370490</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4848,17 +4824,17 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786621975</t>
+          <t>1786623012</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>1786892400</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>146.95082</t>
+          <t>6.980803</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4875,7 +4851,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
+          <t>0xddff1b4ca7359c6045ede1bd2995e1e57620811dc33cc7338113c5449dccd695</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4886,17 +4862,17 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>27.87224</t>
+          <t>28.91904</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.5325</t>
+          <t>1.6038</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -4907,27 +4883,27 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Celta de Vigo vs Osasuna</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Celta de Vigo</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+          <t>0xf684bc2655869d0024c7de5a1f2b51fb35813185b075bf3cc8d5f2fe8ce176b5</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>L19370496</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -4952,17 +4928,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786619056</t>
+          <t>1786622982</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>1786908600</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>52.342235</t>
+          <t>47.899031</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -4979,39 +4955,31 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+          <t>0xb02e365f47ba9eaba62de63e4b14c94bf1b59d60c56188857359df36e7b10ef0</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>30.81465</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.7113</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Rayo Vallecano</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>La Liga</t>
@@ -5019,27 +4987,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Sevilla vs Rayo Vallecano</t>
+          <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Deportivo Alaves</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+          <t>0x8791bf3272cd82404ef50845fa5ccbf5ded7fb2a083138dbf01a1443c1054c54</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>L19370582</t>
+          <t>L19370598</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5064,17 +5032,17 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786614389</t>
+          <t>1786622982</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>1786822200</t>
+          <t>1786815000</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>175.438596</t>
+          <t>43.32464</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5091,12 +5059,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+          <t>0xb7f333fbe5a18daf831395020096fbb62febd43977f5f81366c99339b63d902d</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5106,22 +5074,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>63.86</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.4187</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>La Liga</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -5131,27 +5099,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Deportivo Alaves vs Getafe</t>
+          <t>Racing Santander vs Villarreal</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Deportivo Alaves</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+          <t>0x1518c9a8caca0376f881601c848e03d81cd65f5d32c2b63a51625351cc193e86</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>L19370598</t>
+          <t>L19370490</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5176,17 +5144,17 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786586644</t>
+          <t>1786621976</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1786815000</t>
+          <t>1786892400</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>7.769231</t>
+          <t>152.501493</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5203,102 +5171,766 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>0x79454b5fc310a342a5ad62ccf677e7ea1c42b0e701cd313d0019ee8ec1faf7a2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>97.87</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.305</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0xf9063ec13eee8f96a20b89bd687d0a5f1a3197a4408eb58240f63d72be7c644f</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>320.885246</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0x6df789a868c08b6d011dc9dc3fe38cf8be42973ee6e2b3513f1ae98f3a70e174</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>82.86999</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.7363</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Racing Santander +1</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0xeffd773f9a996fcdab4f40cb833c6db488621204b6af7959d07794c43de040c4</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>112.556862</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x4061873586e14d63aeb0e4cdf23afafe5cd7b3c74fe59157daf06c85b8fd8796</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>44.82</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.305</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Racing Santander -0.5</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Villarreal</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0xb811d0e9d1802cd3762a57ca8fc3a5399392dd37dec4f8d9fd37f0170ece0f50</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19370490</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1786621975</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1786892400</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>146.95082</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0x8dda40aa7d3c4140b3e5ab6ab62f3db4f5a3730a15ebff80f0bda9807c704ca2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>27.87224</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.5325</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Celta de Vigo vs Osasuna</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Celta de Vigo</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x0f075dae0a586d46b2073e126cbc52393dc2ff99a26953308f94b3b2751764b7</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19370496</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1786619056</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1786908600</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>52.342235</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0x4565877a70aabfac9d4d4a2afcda9ace6e304d9bd921ce69a2149c76528e271a</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0xb363112BA7ed93A221Efb405496e4Fa3BE119D81</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Sevilla vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0x2b9c4f75049808a8d2b353d1c6e902da151d2fea092e70f08cdd4ac2ffbfd8a6</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19370582</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1786614389</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1786822200</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>175.438596</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0x562837a4689bf537ab0502cfe5d722bafc1833bc972e329ba5399cd7649a219c</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>La Liga</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves vs Getafe</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Deportivo Alaves</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>0xda132f38d7cbcb404e0db6126292d55c3614e3311c2670ac15890a14a94cdaea</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>L19370598</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1786586644</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>1786815000</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>7.769231</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>0x27be56be09649bd460766fe27df249788cf4d7ad87d19f5f9a8bfba225e519b9</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr">
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
         <is>
           <t>1.52676</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>1.7512</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
         <is>
           <t>La Liga</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Deportivo Alaves vs Getafe</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>Deportivo Alaves</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Getafe</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>0x32766ed977cae312bdb45c44b07e70207b356db986ef0293796496f193e13d1e</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>L19370598</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
         <is>
           <t>1786578252</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>1786815000</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T52" t="inlineStr">
         <is>
           <t>2.032293</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="V52" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>